<commit_message>
Exam Excel : submitted
</commit_message>
<xml_diff>
--- a/Exam/Excel/assessment_project/Data_Analyst_Technical_Assessment_Template.xlsx
+++ b/Exam/Excel/assessment_project/Data_Analyst_Technical_Assessment_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\Project\Data-Analyst\Exam\Excel\assessment_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9660A7-5A95-4044-8E1C-39CA3FCE58AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D09C224-A4DE-4CAC-8AAE-88752E472E21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions &amp; Info" sheetId="1" r:id="rId1"/>
@@ -537,11 +537,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="\R\p\ #,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0\ &quot;Bulan&quot;"/>
     <numFmt numFmtId="167" formatCode="&quot;Rp&quot;#,##0"/>
+    <numFmt numFmtId="168" formatCode="&quot;Rp&quot;#,##0.0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -668,7 +669,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -719,14 +720,17 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1050,75 +1054,75 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
     </row>
     <row r="6" spans="1:8" ht="16.5">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="16.5">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="16.5">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1311,7 +1315,7 @@
     <col min="23" max="23" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="66">
+    <row r="1" spans="1:23" ht="49.5">
       <c r="A1" s="11" t="s">
         <v>29</v>
       </c>
@@ -1428,7 +1432,7 @@
         <f>VLOOKUP(K2,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O2" s="22">
+      <c r="O2" s="20">
         <f>VLOOKUP(K2,Master_Product!$A$2:$D$6,4,0)</f>
         <v>150000</v>
       </c>
@@ -1441,26 +1445,26 @@
         <v>16</v>
       </c>
       <c r="R2" s="10">
-        <f>IF(H2="DISC10",0.1,IF(H2="CASHBACK",0.05,"-"))</f>
+        <f>IF(H2="DISC10",0.1,IF(H2="CASHBACK",0.05,P2))</f>
         <v>0.1</v>
       </c>
       <c r="S2" s="5" t="str">
         <f>IF(Q2&gt;24,"VIP Tier",IF(24&gt;Q2&gt;12,"GOLD Tier","SILVER Tier"))</f>
         <v>GOLD Tier</v>
       </c>
-      <c r="T2" s="22">
+      <c r="T2" s="20">
         <f>O2*G2</f>
         <v>300000</v>
       </c>
-      <c r="U2" s="10">
-        <f>SUM(P2,R2)</f>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V2" s="22">
-        <f>T2-(U2*T2)</f>
-        <v>255000</v>
-      </c>
-      <c r="W2" s="23"/>
+      <c r="U2" s="24">
+        <f>T2*R2</f>
+        <v>30000</v>
+      </c>
+      <c r="V2" s="20">
+        <f>T2-U2</f>
+        <v>270000</v>
+      </c>
+      <c r="W2" s="21"/>
     </row>
     <row r="3" spans="1:23">
       <c r="A3" s="5" t="s">
@@ -1511,7 +1515,7 @@
         <f>VLOOKUP(K3,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Electronics</v>
       </c>
-      <c r="O3" s="22">
+      <c r="O3" s="20">
         <f>VLOOKUP(K3,Master_Product!$A$2:$D$6,4,0)</f>
         <v>250000</v>
       </c>
@@ -1523,24 +1527,24 @@
         <f t="shared" ref="Q3:Q16" si="4">DATEDIF(D3,E3,"M")</f>
         <v>24</v>
       </c>
-      <c r="R3" s="10" t="str">
-        <f t="shared" ref="R3:R16" si="5">IF(H3="DISC10",0.1,IF(H3="CASHBACK",0.05,"-"))</f>
-        <v>-</v>
+      <c r="R3" s="10">
+        <f>IF(H3="DISC10",0.1,IF(H3="CASHBACK",0.05,P3))</f>
+        <v>0.1</v>
       </c>
       <c r="S3" s="5" t="str">
-        <f t="shared" ref="S3:S16" si="6">IF(Q3&gt;24,"VIP Tier",IF(24&gt;Q3&gt;12,"GOLD Tier","SILVER Tier"))</f>
+        <f t="shared" ref="S3:S16" si="5">IF(Q3&gt;24,"VIP Tier",IF(24&gt;Q3&gt;12,"GOLD Tier","SILVER Tier"))</f>
         <v>GOLD Tier</v>
       </c>
-      <c r="T3" s="22">
-        <f t="shared" ref="T3:T16" si="7">O3*G3</f>
+      <c r="T3" s="20">
+        <f t="shared" ref="T3:T16" si="6">O3*G3</f>
         <v>250000</v>
       </c>
-      <c r="U3" s="10">
-        <f t="shared" ref="U3:U16" si="8">SUM(P3,R3)</f>
-        <v>0.1</v>
-      </c>
-      <c r="V3" s="22">
-        <f t="shared" ref="V3:V16" si="9">T3-(U3*T3)</f>
+      <c r="U3" s="24">
+        <f t="shared" ref="U3:U16" si="7">T3*R3</f>
+        <v>25000</v>
+      </c>
+      <c r="V3" s="20">
+        <f t="shared" ref="V3:V16" si="8">T3-U3</f>
         <v>225000</v>
       </c>
     </row>
@@ -1593,7 +1597,7 @@
         <f>VLOOKUP(K4,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Electronics</v>
       </c>
-      <c r="O4" s="22">
+      <c r="O4" s="20">
         <f>VLOOKUP(K4,Master_Product!$A$2:$D$6,4,0)</f>
         <v>750000</v>
       </c>
@@ -1606,24 +1610,24 @@
         <v>5</v>
       </c>
       <c r="R4" s="10">
+        <f t="shared" ref="R4:R16" si="9">IF(H4="DISC10",0.1,IF(H4="CASHBACK",0.05,P4))</f>
+        <v>0.05</v>
+      </c>
+      <c r="S4" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.05</v>
-      </c>
-      <c r="S4" s="5" t="str">
+        <v>GOLD Tier</v>
+      </c>
+      <c r="T4" s="20">
         <f t="shared" si="6"/>
-        <v>GOLD Tier</v>
-      </c>
-      <c r="T4" s="22">
+        <v>3750000</v>
+      </c>
+      <c r="U4" s="24">
         <f t="shared" si="7"/>
-        <v>3750000</v>
-      </c>
-      <c r="U4" s="10">
+        <v>187500</v>
+      </c>
+      <c r="V4" s="20">
         <f t="shared" si="8"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V4" s="22">
-        <f t="shared" si="9"/>
-        <v>3187500</v>
+        <v>3562500</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -1675,7 +1679,7 @@
         <f>VLOOKUP(K5,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O5" s="22">
+      <c r="O5" s="20">
         <f>VLOOKUP(K5,Master_Product!$A$2:$D$6,4,0)</f>
         <v>150000</v>
       </c>
@@ -1688,24 +1692,24 @@
         <v>30</v>
       </c>
       <c r="R5" s="10">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="S5" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.1</v>
-      </c>
-      <c r="S5" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T5" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T5" s="22">
+        <v>150000</v>
+      </c>
+      <c r="U5" s="24">
         <f t="shared" si="7"/>
-        <v>150000</v>
-      </c>
-      <c r="U5" s="10">
+        <v>15000</v>
+      </c>
+      <c r="V5" s="20">
         <f t="shared" si="8"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V5" s="22">
-        <f t="shared" si="9"/>
-        <v>127500</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="6" spans="1:23">
@@ -1757,7 +1761,7 @@
         <f>VLOOKUP(K6,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O6" s="22">
+      <c r="O6" s="20">
         <f>VLOOKUP(K6,Master_Product!$A$2:$D$6,4,0)</f>
         <v>320000</v>
       </c>
@@ -1769,24 +1773,24 @@
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="R6" s="10" t="str">
+      <c r="R6" s="10">
+        <f t="shared" si="9"/>
+        <v>0.05</v>
+      </c>
+      <c r="S6" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-      <c r="S6" s="5" t="str">
+        <v>GOLD Tier</v>
+      </c>
+      <c r="T6" s="20">
         <f t="shared" si="6"/>
-        <v>GOLD Tier</v>
-      </c>
-      <c r="T6" s="22">
+        <v>960000</v>
+      </c>
+      <c r="U6" s="24">
         <f t="shared" si="7"/>
-        <v>960000</v>
-      </c>
-      <c r="U6" s="10">
+        <v>48000</v>
+      </c>
+      <c r="V6" s="20">
         <f t="shared" si="8"/>
-        <v>0.05</v>
-      </c>
-      <c r="V6" s="22">
-        <f t="shared" si="9"/>
         <v>912000</v>
       </c>
     </row>
@@ -1839,7 +1843,7 @@
         <f>VLOOKUP(K7,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Electronics</v>
       </c>
-      <c r="O7" s="22">
+      <c r="O7" s="20">
         <f>VLOOKUP(K7,Master_Product!$A$2:$D$6,4,0)</f>
         <v>250000</v>
       </c>
@@ -1852,24 +1856,24 @@
         <v>51</v>
       </c>
       <c r="R7" s="10">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="S7" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.1</v>
-      </c>
-      <c r="S7" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T7" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T7" s="22">
+        <v>1000000</v>
+      </c>
+      <c r="U7" s="24">
         <f t="shared" si="7"/>
-        <v>1000000</v>
-      </c>
-      <c r="U7" s="10">
+        <v>100000</v>
+      </c>
+      <c r="V7" s="20">
         <f t="shared" si="8"/>
-        <v>0.2</v>
-      </c>
-      <c r="V7" s="22">
-        <f t="shared" si="9"/>
-        <v>800000</v>
+        <v>900000</v>
       </c>
     </row>
     <row r="8" spans="1:23">
@@ -1921,7 +1925,7 @@
         <f>VLOOKUP(K8,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Furniture</v>
       </c>
-      <c r="O8" s="22">
+      <c r="O8" s="20">
         <f>VLOOKUP(K8,Master_Product!$A$2:$D$6,4,0)</f>
         <v>450000</v>
       </c>
@@ -1934,24 +1938,24 @@
         <v>28</v>
       </c>
       <c r="R8" s="10">
+        <f t="shared" si="9"/>
+        <v>0.05</v>
+      </c>
+      <c r="S8" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.05</v>
-      </c>
-      <c r="S8" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T8" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T8" s="22">
+        <v>900000</v>
+      </c>
+      <c r="U8" s="24">
         <f t="shared" si="7"/>
-        <v>900000</v>
-      </c>
-      <c r="U8" s="10">
+        <v>45000</v>
+      </c>
+      <c r="V8" s="20">
         <f t="shared" si="8"/>
-        <v>0.13</v>
-      </c>
-      <c r="V8" s="22">
-        <f t="shared" si="9"/>
-        <v>783000</v>
+        <v>855000</v>
       </c>
     </row>
     <row r="9" spans="1:23">
@@ -2003,7 +2007,7 @@
         <f>VLOOKUP(K9,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O9" s="22">
+      <c r="O9" s="20">
         <f>VLOOKUP(K9,Master_Product!$A$2:$D$6,4,0)</f>
         <v>150000</v>
       </c>
@@ -2015,24 +2019,24 @@
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="R9" s="10" t="str">
+      <c r="R9" s="10">
+        <f t="shared" si="9"/>
+        <v>0.05</v>
+      </c>
+      <c r="S9" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-      <c r="S9" s="5" t="str">
+        <v>GOLD Tier</v>
+      </c>
+      <c r="T9" s="20">
         <f t="shared" si="6"/>
-        <v>GOLD Tier</v>
-      </c>
-      <c r="T9" s="22">
+        <v>150000</v>
+      </c>
+      <c r="U9" s="24">
         <f t="shared" si="7"/>
-        <v>150000</v>
-      </c>
-      <c r="U9" s="10">
+        <v>7500</v>
+      </c>
+      <c r="V9" s="20">
         <f t="shared" si="8"/>
-        <v>0.05</v>
-      </c>
-      <c r="V9" s="22">
-        <f t="shared" si="9"/>
         <v>142500</v>
       </c>
     </row>
@@ -2085,7 +2089,7 @@
         <f>VLOOKUP(K10,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O10" s="22">
+      <c r="O10" s="20">
         <f>VLOOKUP(K10,Master_Product!$A$2:$D$6,4,0)</f>
         <v>320000</v>
       </c>
@@ -2098,24 +2102,24 @@
         <v>37</v>
       </c>
       <c r="R10" s="10">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="S10" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.1</v>
-      </c>
-      <c r="S10" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T10" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T10" s="22">
+        <v>640000</v>
+      </c>
+      <c r="U10" s="24">
         <f t="shared" si="7"/>
-        <v>640000</v>
-      </c>
-      <c r="U10" s="10">
+        <v>64000</v>
+      </c>
+      <c r="V10" s="20">
         <f t="shared" si="8"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V10" s="22">
-        <f t="shared" si="9"/>
-        <v>544000</v>
+        <v>576000</v>
       </c>
     </row>
     <row r="11" spans="1:23">
@@ -2167,7 +2171,7 @@
         <f>VLOOKUP(K11,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Electronics</v>
       </c>
-      <c r="O11" s="22">
+      <c r="O11" s="20">
         <f>VLOOKUP(K11,Master_Product!$A$2:$D$6,4,0)</f>
         <v>750000</v>
       </c>
@@ -2179,24 +2183,24 @@
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="R11" s="10" t="str">
+      <c r="R11" s="10">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="S11" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-      <c r="S11" s="5" t="str">
+        <v>GOLD Tier</v>
+      </c>
+      <c r="T11" s="20">
         <f t="shared" si="6"/>
-        <v>GOLD Tier</v>
-      </c>
-      <c r="T11" s="22">
+        <v>750000</v>
+      </c>
+      <c r="U11" s="24">
         <f t="shared" si="7"/>
-        <v>750000</v>
-      </c>
-      <c r="U11" s="10">
+        <v>75000</v>
+      </c>
+      <c r="V11" s="20">
         <f t="shared" si="8"/>
-        <v>0.1</v>
-      </c>
-      <c r="V11" s="22">
-        <f t="shared" si="9"/>
         <v>675000</v>
       </c>
     </row>
@@ -2249,7 +2253,7 @@
         <f>VLOOKUP(K12,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Electronics</v>
       </c>
-      <c r="O12" s="22">
+      <c r="O12" s="20">
         <f>VLOOKUP(K12,Master_Product!$A$2:$D$6,4,0)</f>
         <v>250000</v>
       </c>
@@ -2262,24 +2266,24 @@
         <v>21</v>
       </c>
       <c r="R12" s="10">
+        <f t="shared" si="9"/>
+        <v>0.05</v>
+      </c>
+      <c r="S12" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.05</v>
-      </c>
-      <c r="S12" s="5" t="str">
+        <v>GOLD Tier</v>
+      </c>
+      <c r="T12" s="20">
         <f t="shared" si="6"/>
-        <v>GOLD Tier</v>
-      </c>
-      <c r="T12" s="22">
+        <v>750000</v>
+      </c>
+      <c r="U12" s="24">
         <f t="shared" si="7"/>
-        <v>750000</v>
-      </c>
-      <c r="U12" s="10">
+        <v>37500</v>
+      </c>
+      <c r="V12" s="20">
         <f t="shared" si="8"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V12" s="22">
-        <f t="shared" si="9"/>
-        <v>637500</v>
+        <v>712500</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -2331,7 +2335,7 @@
         <f>VLOOKUP(K13,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Furniture</v>
       </c>
-      <c r="O13" s="22">
+      <c r="O13" s="20">
         <f>VLOOKUP(K13,Master_Product!$A$2:$D$6,4,0)</f>
         <v>450000</v>
       </c>
@@ -2344,24 +2348,24 @@
         <v>47</v>
       </c>
       <c r="R13" s="10">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="S13" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.1</v>
-      </c>
-      <c r="S13" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T13" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T13" s="22">
+        <v>450000</v>
+      </c>
+      <c r="U13" s="24">
         <f t="shared" si="7"/>
-        <v>450000</v>
-      </c>
-      <c r="U13" s="10">
+        <v>45000</v>
+      </c>
+      <c r="V13" s="20">
         <f t="shared" si="8"/>
-        <v>0.18</v>
-      </c>
-      <c r="V13" s="22">
-        <f t="shared" si="9"/>
-        <v>369000</v>
+        <v>405000</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -2413,7 +2417,7 @@
         <f>VLOOKUP(K14,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O14" s="22">
+      <c r="O14" s="20">
         <f>VLOOKUP(K14,Master_Product!$A$2:$D$6,4,0)</f>
         <v>150000</v>
       </c>
@@ -2425,24 +2429,24 @@
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="R14" s="10" t="str">
+      <c r="R14" s="10">
+        <f t="shared" si="9"/>
+        <v>0.05</v>
+      </c>
+      <c r="S14" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-      <c r="S14" s="5" t="str">
+        <v>GOLD Tier</v>
+      </c>
+      <c r="T14" s="20">
         <f t="shared" si="6"/>
-        <v>GOLD Tier</v>
-      </c>
-      <c r="T14" s="22">
+        <v>300000</v>
+      </c>
+      <c r="U14" s="24">
         <f t="shared" si="7"/>
-        <v>300000</v>
-      </c>
-      <c r="U14" s="10">
+        <v>15000</v>
+      </c>
+      <c r="V14" s="20">
         <f t="shared" si="8"/>
-        <v>0.05</v>
-      </c>
-      <c r="V14" s="22">
-        <f t="shared" si="9"/>
         <v>285000</v>
       </c>
     </row>
@@ -2495,7 +2499,7 @@
         <f>VLOOKUP(K15,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Accessories</v>
       </c>
-      <c r="O15" s="22">
+      <c r="O15" s="20">
         <f>VLOOKUP(K15,Master_Product!$A$2:$D$6,4,0)</f>
         <v>320000</v>
       </c>
@@ -2508,24 +2512,24 @@
         <v>29</v>
       </c>
       <c r="R15" s="10">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="S15" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.1</v>
-      </c>
-      <c r="S15" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T15" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T15" s="22">
+        <v>1280000</v>
+      </c>
+      <c r="U15" s="24">
         <f t="shared" si="7"/>
-        <v>1280000</v>
-      </c>
-      <c r="U15" s="10">
+        <v>128000</v>
+      </c>
+      <c r="V15" s="20">
         <f t="shared" si="8"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V15" s="22">
-        <f t="shared" si="9"/>
-        <v>1088000</v>
+        <v>1152000</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -2577,7 +2581,7 @@
         <f>VLOOKUP(K16,Master_Product!$A$2:$D$6,3,FALSE)</f>
         <v>Electronics</v>
       </c>
-      <c r="O16" s="22">
+      <c r="O16" s="20">
         <f>VLOOKUP(K16,Master_Product!$A$2:$D$6,4,0)</f>
         <v>750000</v>
       </c>
@@ -2590,24 +2594,24 @@
         <v>56</v>
       </c>
       <c r="R16" s="10">
+        <f t="shared" si="9"/>
+        <v>0.05</v>
+      </c>
+      <c r="S16" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>0.05</v>
-      </c>
-      <c r="S16" s="5" t="str">
+        <v>VIP Tier</v>
+      </c>
+      <c r="T16" s="20">
         <f t="shared" si="6"/>
-        <v>VIP Tier</v>
-      </c>
-      <c r="T16" s="22">
+        <v>1500000</v>
+      </c>
+      <c r="U16" s="24">
         <f t="shared" si="7"/>
-        <v>1500000</v>
-      </c>
-      <c r="U16" s="10">
+        <v>75000</v>
+      </c>
+      <c r="V16" s="20">
         <f t="shared" si="8"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="V16" s="22">
-        <f t="shared" si="9"/>
-        <v>1275000</v>
+        <v>1425000</v>
       </c>
     </row>
   </sheetData>
@@ -2659,7 +2663,7 @@
       </c>
       <c r="B5" s="7">
         <f>SUM(Raw_Transactions!V2:V16)</f>
-        <v>11306000</v>
+        <v>12232500</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>144</v>
@@ -2670,8 +2674,8 @@
         <v>146</v>
       </c>
       <c r="B6" s="7">
-        <f>SUM(Raw_Transactions!U2:U16)</f>
-        <v>1.9100000000000001</v>
+        <f>SUM(B4-B5)</f>
+        <v>897500</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>144</v>
@@ -2681,7 +2685,10 @@
       <c r="A7" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B7" s="18"/>
+      <c r="B7" s="18">
+        <f>COUNTA(Raw_Transactions!G2:G16)</f>
+        <v>15</v>
+      </c>
       <c r="C7" s="5" t="s">
         <v>148</v>
       </c>
@@ -2690,7 +2697,10 @@
       <c r="A8" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="B8" s="18"/>
+      <c r="B8" s="18">
+        <f>SUM(Raw_Transactions!G2:G16)</f>
+        <v>34</v>
+      </c>
       <c r="C8" s="5" t="s">
         <v>144</v>
       </c>
@@ -2699,7 +2709,10 @@
       <c r="A9" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="7">
+        <f>AVERAGE(Raw_Transactions!T2:T16)</f>
+        <v>875333.33333333337</v>
+      </c>
       <c r="C9" s="5" t="s">
         <v>151</v>
       </c>
@@ -2708,7 +2721,10 @@
       <c r="A10" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="B10" s="7"/>
+      <c r="B10" s="7">
+        <f>AVERAGE(Raw_Transactions!V2:V16)</f>
+        <v>815500</v>
+      </c>
       <c r="C10" s="5" t="s">
         <v>151</v>
       </c>
@@ -2717,7 +2733,10 @@
       <c r="A11" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="7">
+        <f>MAX(Raw_Transactions!T2:T16)</f>
+        <v>3750000</v>
+      </c>
       <c r="C11" s="5" t="s">
         <v>154</v>
       </c>
@@ -2726,7 +2745,10 @@
       <c r="A12" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="B12" s="7"/>
+      <c r="B12" s="7">
+        <f>MIN(Raw_Transactions!T2:T16)</f>
+        <v>150000</v>
+      </c>
       <c r="C12" s="5" t="s">
         <v>156</v>
       </c>
@@ -2735,7 +2757,10 @@
       <c r="A13" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="B13" s="19"/>
+      <c r="B13" s="19">
+        <f>AVERAGE(Raw_Transactions!Q2:Q16)</f>
+        <v>25.2</v>
+      </c>
       <c r="C13" s="5" t="s">
         <v>151</v>
       </c>

</xml_diff>